<commit_message>
chore(matrix): actualizar conteo de jobs (7→10) y registrar 11 commits nuevos
generar-matriz-registro.py:
- INT-003-BOLT-001, ART-006, PMV-008, P-009, BPMN task:
  "6/7 jobs" → "10 jobs" con lista completa (bdd, k6-smoke, lighthouse).
- COMMITS: añade 11 entradas 05/2026–06/2026 (flutter tests, k6, lighthouse,
  bdd, handleSummary, docs 422→507, matrix 100%, CI SLA).
  Total registrados: 25 → 36.

apply_aidlc.py:
- INT-003-001 evidencia: "6 jobs" → "10 jobs con timeout-minutes".

Excel: regenerado (Commits registrados: 36, Avance: 100.0%).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/matriz-registro-hearguard.xlsx
+++ b/docs/matriz-registro-hearguard.xlsx
@@ -1779,7 +1779,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Versión 4.0  ·  Generada: 10/06/2026 00:09  ·  2026-I</t>
+          <t>Versión 4.0  ·  Generada: 10/06/2026 00:13  ·  2026-I</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2301,7 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>25 commits</t>
+          <t>36 commits</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>25 eventos</t>
+          <t>36 eventos</t>
         </is>
       </c>
     </row>
@@ -2939,7 +2939,7 @@
       </c>
       <c r="H12" s="47" t="inlineStr">
         <is>
-          <t>GitHub Actions: 7 jobs (backend, ai-service, frontend, e2e, flutter, sonar, deploy)</t>
+          <t>GitHub Actions: 10 jobs (backend, ai-service, frontend, bdd, e2e, flutter, sonarcloud, k6-smoke, lighthouse, deploy)</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3664,7 @@
       </c>
       <c r="F14" s="47" t="inlineStr">
         <is>
-          <t>7 jobs: backend, ai, frontend, e2e, flutter, sonar, deploy</t>
+          <t>10 jobs: backend, ai, frontend, bdd, e2e, flutter, sonar, k6-smoke, lighthouse, deploy</t>
         </is>
       </c>
       <c r="G14" s="47" t="inlineStr">
@@ -9433,7 +9433,7 @@
       </c>
       <c r="H19" s="47" t="inlineStr">
         <is>
-          <t>03–05/2026</t>
+          <t>03–06/2026</t>
         </is>
       </c>
       <c r="I19" s="47" t="inlineStr">
@@ -9473,7 +9473,7 @@
       </c>
       <c r="P19" s="47" t="inlineStr">
         <is>
-          <t>ci.yml</t>
+          <t>ci.yml — 10 jobs con timeout-minutes</t>
         </is>
       </c>
     </row>
@@ -12297,7 +12297,7 @@
       </c>
       <c r="I20" s="47" t="inlineStr">
         <is>
-          <t>03–05/2026</t>
+          <t>03–06/2026</t>
         </is>
       </c>
     </row>
@@ -13773,7 +13773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14882,6 +14882,468 @@
       <c r="H28" s="50" t="inlineStr">
         <is>
           <t>[13cdf60] fix(ci): fix gen-flutter-lock workflow token + git add path</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>MRG-026</t>
+        </is>
+      </c>
+      <c r="B29" s="114" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="C29" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D29" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E29" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="F29" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G29" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H29" s="50" t="inlineStr">
+        <is>
+          <t>[b012733] test(flutter): añadir 22 tests + fix score_to_years determin</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="47" t="inlineStr">
+        <is>
+          <t>MRG-027</t>
+        </is>
+      </c>
+      <c r="B30" s="118" t="inlineStr">
+        <is>
+          <t>ci</t>
+        </is>
+      </c>
+      <c r="C30" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D30" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E30" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="F30" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G30" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H30" s="50" t="inlineStr">
+        <is>
+          <t>[945cccd] ci(k6): agregar job smoke de performance en CI post-deploy</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>MRG-028</t>
+        </is>
+      </c>
+      <c r="B31" s="122" t="inlineStr">
+        <is>
+          <t>refactor</t>
+        </is>
+      </c>
+      <c r="C31" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D31" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E31" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G31" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H31" s="50" t="inlineStr">
+        <is>
+          <t>[228a21e] refactor(frontend): extraer estilos inline a archivos .compo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="47" t="inlineStr">
+        <is>
+          <t>MRG-029</t>
+        </is>
+      </c>
+      <c r="B32" s="118" t="inlineStr">
+        <is>
+          <t>ci</t>
+        </is>
+      </c>
+      <c r="C32" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D32" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E32" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="F32" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G32" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H32" s="50" t="inlineStr">
+        <is>
+          <t>[0527cd5] ci(lighthouse): agregar job de auditoría de performance Ligh</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>MRG-030</t>
+        </is>
+      </c>
+      <c r="B33" s="118" t="inlineStr">
+        <is>
+          <t>ci</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E33" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G33" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H33" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[27bef44] ci(bdd): agregar ejecución automática de escenarios Gherkin </t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="47" t="inlineStr">
+        <is>
+          <t>MRG-031</t>
+        </is>
+      </c>
+      <c r="B34" s="118" t="inlineStr">
+        <is>
+          <t>ci</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E34" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G34" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H34" s="50" t="inlineStr">
+        <is>
+          <t>[672ece3] ci(k6): generar reporte HTML con handleSummary en producción</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="47" t="inlineStr">
+        <is>
+          <t>MRG-032</t>
+        </is>
+      </c>
+      <c r="B35" s="120" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G35" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H35" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[18fd16e] docs(articulo): actualizar métricas y limitaciones tras BDD </t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>MRG-033</t>
+        </is>
+      </c>
+      <c r="B36" s="120" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E36" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G36" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H36" s="50" t="inlineStr">
+        <is>
+          <t>[c8d3f7a] docs: sincronizar metodologia y plan-de-pruebas con estado r</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>MRG-034</t>
+        </is>
+      </c>
+      <c r="B37" s="120" t="inlineStr">
+        <is>
+          <t>docs</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E37" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G37" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H37" s="50" t="inlineStr">
+        <is>
+          <t>[3a8bb79] docs: actualizar 422 → 507 en toda la documentación académic</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="47" t="inlineStr">
+        <is>
+          <t>MRG-035</t>
+        </is>
+      </c>
+      <c r="B38" s="125" t="inlineStr">
+        <is>
+          <t>chore</t>
+        </is>
+      </c>
+      <c r="C38" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D38" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E38" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="F38" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G38" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H38" s="50" t="inlineStr">
+        <is>
+          <t>[6f8b169] chore(matrix): marcar bolts BDD/k6/Lighthouse como completad</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="47" t="inlineStr">
+        <is>
+          <t>MRG-036</t>
+        </is>
+      </c>
+      <c r="B39" s="118" t="inlineStr">
+        <is>
+          <t>ci</t>
+        </is>
+      </c>
+      <c r="C39" s="47" t="inlineStr">
+        <is>
+          <t>feature/fix</t>
+        </is>
+      </c>
+      <c r="D39" s="47" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E39" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="F39" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+      <c r="G39" s="115" t="inlineStr">
+        <is>
+          <t>Integrado</t>
+        </is>
+      </c>
+      <c r="H39" s="50" t="inlineStr">
+        <is>
+          <t>[1e56763] ci(sla): agregar timeout-minutes y npm audit al pipeline</t>
         </is>
       </c>
     </row>
@@ -14916,6 +15378,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14927,7 +15400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15903,6 +16376,413 @@
         </is>
       </c>
       <c r="G28" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B29" s="50" t="inlineStr">
+        <is>
+          <t>commit:b012733</t>
+        </is>
+      </c>
+      <c r="C29" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D29" s="114" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="E29" s="47" t="inlineStr">
+        <is>
+          <t>test(flutter): añadir 22 tests + fix score_to_years determinista</t>
+        </is>
+      </c>
+      <c r="F29" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G29" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B30" s="50" t="inlineStr">
+        <is>
+          <t>commit:945cccd</t>
+        </is>
+      </c>
+      <c r="C30" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D30" s="118" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E30" s="47" t="inlineStr">
+        <is>
+          <t>ci(k6): agregar job smoke de performance en CI post-deploy</t>
+        </is>
+      </c>
+      <c r="F30" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G30" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B31" s="50" t="inlineStr">
+        <is>
+          <t>commit:228a21e</t>
+        </is>
+      </c>
+      <c r="C31" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D31" s="122" t="inlineStr">
+        <is>
+          <t>REFACTOR</t>
+        </is>
+      </c>
+      <c r="E31" s="47" t="inlineStr">
+        <is>
+          <t>refactor(frontend): extraer estilos inline a archivos .component.scss</t>
+        </is>
+      </c>
+      <c r="F31" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G31" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="47" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B32" s="50" t="inlineStr">
+        <is>
+          <t>commit:0527cd5</t>
+        </is>
+      </c>
+      <c r="C32" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D32" s="118" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E32" s="47" t="inlineStr">
+        <is>
+          <t>ci(lighthouse): agregar job de auditoría de performance Lighthouse en Vercel</t>
+        </is>
+      </c>
+      <c r="F32" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G32" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B33" s="50" t="inlineStr">
+        <is>
+          <t>commit:27bef44</t>
+        </is>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D33" s="118" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E33" s="47" t="inlineStr">
+        <is>
+          <t>ci(bdd): agregar ejecución automática de escenarios Gherkin con Cucumber.js</t>
+        </is>
+      </c>
+      <c r="F33" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G33" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B34" s="50" t="inlineStr">
+        <is>
+          <t>commit:672ece3</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D34" s="118" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E34" s="47" t="inlineStr">
+        <is>
+          <t>ci(k6): generar reporte HTML con handleSummary en producción</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G34" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="inlineStr">
+        <is>
+          <t>commit:18fd16e</t>
+        </is>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D35" s="120" t="inlineStr">
+        <is>
+          <t>DOCS</t>
+        </is>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>docs(articulo): actualizar métricas y limitaciones tras BDD + k6 HTML</t>
+        </is>
+      </c>
+      <c r="F35" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G35" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B36" s="50" t="inlineStr">
+        <is>
+          <t>commit:c8d3f7a</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D36" s="120" t="inlineStr">
+        <is>
+          <t>DOCS</t>
+        </is>
+      </c>
+      <c r="E36" s="47" t="inlineStr">
+        <is>
+          <t>docs: sincronizar metodologia y plan-de-pruebas con estado real del repo</t>
+        </is>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G36" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B37" s="50" t="inlineStr">
+        <is>
+          <t>commit:3a8bb79</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D37" s="120" t="inlineStr">
+        <is>
+          <t>DOCS</t>
+        </is>
+      </c>
+      <c r="E37" s="47" t="inlineStr">
+        <is>
+          <t>docs: actualizar 422 → 507 en toda la documentación académica</t>
+        </is>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G37" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B38" s="50" t="inlineStr">
+        <is>
+          <t>commit:6f8b169</t>
+        </is>
+      </c>
+      <c r="C38" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D38" s="125" t="inlineStr">
+        <is>
+          <t>CHORE</t>
+        </is>
+      </c>
+      <c r="E38" s="47" t="inlineStr">
+        <is>
+          <t>chore(matrix): marcar bolts BDD/k6/Lighthouse como completados; avance 97.5%</t>
+        </is>
+      </c>
+      <c r="F38" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G38" s="47" t="inlineStr">
+        <is>
+          <t>Luis F. Terreros H.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="47" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B39" s="50" t="inlineStr">
+        <is>
+          <t>commit:1e56763</t>
+        </is>
+      </c>
+      <c r="C39" s="47" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="D39" s="118" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="E39" s="47" t="inlineStr">
+        <is>
+          <t>ci(sla): agregar timeout-minutes y npm audit al pipeline</t>
+        </is>
+      </c>
+      <c r="F39" s="47" t="inlineStr">
+        <is>
+          <t>Claude Sonnet</t>
+        </is>
+      </c>
+      <c r="G39" s="47" t="inlineStr">
         <is>
           <t>Luis F. Terreros H.</t>
         </is>
@@ -15939,6 +16819,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16224,7 +17115,7 @@
       </c>
       <c r="G9" s="47" t="inlineStr">
         <is>
-          <t>7 jobs: backend, ai-service, frontend, e2e, flutter, sonarcloud, deploy</t>
+          <t>10 jobs: backend, ai-service, frontend, bdd, e2e, flutter, sonarcloud, k6-smoke, lighthouse, deploy</t>
         </is>
       </c>
     </row>
@@ -16715,7 +17606,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>Generado: 10/06/2026 00:09  ·  Autor: Luis Francisco Terreros Hinojosa  ·  Universidad Continental</t>
+          <t>Generado: 10/06/2026 00:13  ·  Autor: Luis Francisco Terreros Hinojosa  ·  Universidad Continental</t>
         </is>
       </c>
     </row>
@@ -16825,7 +17716,7 @@
       </c>
       <c r="I5" s="23" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>36</t>
         </is>
       </c>
       <c r="J5" s="23" t="inlineStr">
@@ -18100,7 +18991,7 @@
       </c>
       <c r="F12" s="47" t="inlineStr">
         <is>
-          <t>7 jobs automatizados: test + lint + coverage + sonarcloud + deploy</t>
+          <t>10 jobs: backend, ai-service, frontend, bdd, e2e, flutter, sonarcloud, k6-smoke, lighthouse, deploy</t>
         </is>
       </c>
     </row>
@@ -18416,7 +19307,7 @@
       </c>
       <c r="B20" s="129" t="inlineStr">
         <is>
-          <t>25 commits a main con fecha, hash y enlace a GitHub</t>
+          <t>36 commits a main con fecha, hash y enlace a GitHub</t>
         </is>
       </c>
     </row>
@@ -18428,7 +19319,7 @@
       </c>
       <c r="B21" s="129" t="inlineStr">
         <is>
-          <t>Log cronológico de 25 cambios del proyecto</t>
+          <t>Log cronológico de 36 cambios del proyecto</t>
         </is>
       </c>
     </row>
@@ -19691,7 +20582,7 @@
       </c>
       <c r="C21" s="47" t="inlineStr">
         <is>
-          <t>Jobs: backend, ai-service, frontend, e2e, flutter, sonarcloud</t>
+          <t>Jobs: backend, ai-service, frontend, bdd, e2e, flutter, sonarcloud, k6-smoke, lighthouse, deploy</t>
         </is>
       </c>
       <c r="D21" s="47" t="inlineStr">
@@ -19701,7 +20592,7 @@
       </c>
       <c r="E21" s="47" t="inlineStr">
         <is>
-          <t>03–05/2026</t>
+          <t>03–06/2026</t>
         </is>
       </c>
       <c r="F21" s="47" t="inlineStr">
@@ -19726,7 +20617,7 @@
       </c>
       <c r="J21" s="47" t="inlineStr">
         <is>
-          <t>ci.yml</t>
+          <t>ci.yml — 10 jobs con timeout-minutes</t>
         </is>
       </c>
       <c r="K21" s="50" t="inlineStr">

</xml_diff>

<commit_message>
docs(readme): actualizar 422→507 y 7→10 jobs en tabla resumen
- README.md: 422 → 507 casos con desglose por capa, CI 7 → 10 jobs
- scripts/generar-matriz-registro.py: label sheet 422→507 tests
- docs/matriz-registro-hearguard.xlsx: regenerado (40/40 Si, 100%)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/matriz-registro-hearguard.xlsx
+++ b/docs/matriz-registro-hearguard.xlsx
@@ -1779,7 +1779,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Versión 4.0  ·  Generada: 10/06/2026 00:13  ·  2026-I</t>
+          <t>Versión 4.0  ·  Generada: 10/06/2026 00:27  ·  2026-I</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>422 tests por capa con comandos de ejecución</t>
+          <t>507 tests por capa con comandos de ejecución</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
@@ -17606,7 +17606,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>Generado: 10/06/2026 00:13  ·  Autor: Luis Francisco Terreros Hinojosa  ·  Universidad Continental</t>
+          <t>Generado: 10/06/2026 00:27  ·  Autor: Luis Francisco Terreros Hinojosa  ·  Universidad Continental</t>
         </is>
       </c>
     </row>

</xml_diff>